<commit_message>
feat(sales): add monthly breakdown sheets to prepaid-MSA workbook (bookings + accrual)
Adds two month-by-month sheets (columns Mo1-12 + Year 1), formula-driven from Assumptions:
- Monthly (Bookings): cash/bookings basis; full annual collected + 15% commission upfront,
  year-end MSA bonus in Mo12; sums to the Full Forecast P&L.
- Monthly (Accrual): GAAP/ASC 606; revenue recognized ratably as cohorts stack, commission
  amortized; shows deferred revenue carried to Yr2.
Workbook now 8 sheets. Updates Documents page description.

Co-authored-by: marcellmiller27 <marcellmiller27@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/JHI_Sales_Commission_Prepaid_MSA.xlsx
+++ b/public/downloads/JHI_Sales_Commission_Prepaid_MSA.xlsx
@@ -11,8 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upfront Commission (15%)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Year-End MSA Bonus" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Forecast P&amp;L" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salesperson Total Comp" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legal &amp; Provenance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly (Bookings)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly (Accrual)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salesperson Total Comp" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legal &amp; Provenance" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -508,7 +510,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>generated 2026-07-18  ·  JHI-SIG: 69M2705M</t>
+          <t>generated 2026-07-19  ·  JHI-SIG: 69M2705M</t>
         </is>
       </c>
     </row>
@@ -809,7 +811,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>generated 2026-07-18  ·  JHI-SIG: 69M2705M</t>
+          <t>generated 2026-07-19  ·  JHI-SIG: 69M2705M</t>
         </is>
       </c>
     </row>
@@ -981,7 +983,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>generated 2026-07-18  ·  JHI-SIG: 69M2705M</t>
+          <t>generated 2026-07-19  ·  JHI-SIG: 69M2705M</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1139,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>generated 2026-07-18  ·  JHI-SIG: 69M2705M</t>
+          <t>generated 2026-07-19  ·  JHI-SIG: 69M2705M</t>
         </is>
       </c>
     </row>
@@ -1344,13 +1346,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1363,197 +1375,857 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Salesperson total compensation &amp; mix sensitivity</t>
+          <t>Monthly breakdown — bookings / cash basis</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>generated 2026-07-18  ·  JHI-SIG: 69M2705M</t>
+          <t>generated 2026-07-19  ·  JHI-SIG: 69M2705M</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Each month books `closes` prepaid annual contracts: full annual value collected + 15% commission paid UP FRONT that month. Year-end MSA bonus in Mo 12. Sums to the P&amp;L.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Upfront commission (15%)</t>
-        </is>
-      </c>
-      <c r="B5" s="15">
-        <f>'Upfront Commission (15%)'!$D$10</f>
-        <v/>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>$ per month</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 1</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 2</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 3</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 4</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 5</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 6</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 7</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 8</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 9</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 10</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 11</t>
+        </is>
+      </c>
+      <c r="M5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 12</t>
+        </is>
+      </c>
+      <c r="N5" s="12" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Year-end MSA-completion bonus</t>
-        </is>
-      </c>
-      <c r="B6" s="15">
-        <f>'Year-End MSA Bonus'!$B$10</f>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>New subscriptions</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="C6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="D6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="E6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="F6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="G6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="H6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="I6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="J6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="K6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="L6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="M6" s="8">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="N6" s="8">
+        <f>SUM(B6:M6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Total salesperson compensation</t>
-        </is>
-      </c>
-      <c r="B7" s="13">
-        <f>B5+B6</f>
+          <t>Revenue (booked)</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="C7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="F7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="G7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="H7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="I7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="J7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="K7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="L7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="M7" s="15">
+        <f>Assumptions!$B$8*Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="N7" s="15">
+        <f>SUM(B7:M7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Total comp as % of revenue</t>
-        </is>
-      </c>
-      <c r="B8" s="14">
-        <f>IF(Assumptions!$B$17=0,0,B7/Assumptions!$B$17)</f>
+          <t xml:space="preserve">  Payment processing</t>
+        </is>
+      </c>
+      <c r="B8" s="9">
+        <f>B7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="C8" s="9">
+        <f>C7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="D8" s="9">
+        <f>D7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="E8" s="9">
+        <f>E7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="F8" s="9">
+        <f>F7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="G8" s="9">
+        <f>G7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="H8" s="9">
+        <f>H7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="I8" s="9">
+        <f>I7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="J8" s="9">
+        <f>J7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="K8" s="9">
+        <f>K7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="L8" s="9">
+        <f>L7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="M8" s="9">
+        <f>M7*Assumptions!$B$20/100</f>
+        <v/>
+      </c>
+      <c r="N8" s="9">
+        <f>SUM(B8:M8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Infrastructure &amp; support</t>
+        </is>
+      </c>
+      <c r="B9" s="9">
+        <f>B7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="C9" s="9">
+        <f>C7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="D9" s="9">
+        <f>D7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="E9" s="9">
+        <f>E7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="F9" s="9">
+        <f>F7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="G9" s="9">
+        <f>G7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="H9" s="9">
+        <f>H7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="I9" s="9">
+        <f>I7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="J9" s="9">
+        <f>J7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="K9" s="9">
+        <f>K7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="L9" s="9">
+        <f>L7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="M9" s="9">
+        <f>M7*Assumptions!$B$21/100</f>
+        <v/>
+      </c>
+      <c r="N9" s="9">
+        <f>SUM(B9:M9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Data license (SF1)</t>
+        </is>
+      </c>
+      <c r="B10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="C10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="D10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="E10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="F10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="G10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="H10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="I10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="J10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="K10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="L10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="M10" s="9">
+        <f>Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="N10" s="9">
+        <f>SUM(B10:M10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Sensitivity — by Tier-1 mix (1,200 subs)</t>
-        </is>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Total COGS</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>SUM(B8:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="9">
+        <f>SUM(C8:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="9">
+        <f>SUM(D8:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="9">
+        <f>SUM(E8:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="9">
+        <f>SUM(F8:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="9">
+        <f>SUM(G8:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="9">
+        <f>SUM(H8:H10)</f>
+        <v/>
+      </c>
+      <c r="I11" s="9">
+        <f>SUM(I8:I10)</f>
+        <v/>
+      </c>
+      <c r="J11" s="9">
+        <f>SUM(J8:J10)</f>
+        <v/>
+      </c>
+      <c r="K11" s="9">
+        <f>SUM(K8:K10)</f>
+        <v/>
+      </c>
+      <c r="L11" s="9">
+        <f>SUM(L8:L10)</f>
+        <v/>
+      </c>
+      <c r="M11" s="9">
+        <f>SUM(M8:M10)</f>
+        <v/>
+      </c>
+      <c r="N11" s="9">
+        <f>SUM(B11:M11)</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>0% T1</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>10% T1</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>20% T1</t>
-        </is>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Gross profit</t>
+        </is>
+      </c>
+      <c r="B12" s="15">
+        <f>B7-B11</f>
+        <v/>
+      </c>
+      <c r="C12" s="15">
+        <f>C7-C11</f>
+        <v/>
+      </c>
+      <c r="D12" s="15">
+        <f>D7-D11</f>
+        <v/>
+      </c>
+      <c r="E12" s="15">
+        <f>E7-E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="15">
+        <f>F7-F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="15">
+        <f>G7-G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="15">
+        <f>H7-H11</f>
+        <v/>
+      </c>
+      <c r="I12" s="15">
+        <f>I7-I11</f>
+        <v/>
+      </c>
+      <c r="J12" s="15">
+        <f>J7-J11</f>
+        <v/>
+      </c>
+      <c r="K12" s="15">
+        <f>K7-K11</f>
+        <v/>
+      </c>
+      <c r="L12" s="15">
+        <f>L7-L11</f>
+        <v/>
+      </c>
+      <c r="M12" s="15">
+        <f>M7-M11</f>
+        <v/>
+      </c>
+      <c r="N12" s="15">
+        <f>SUM(B12:M12)</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Avg full-paid price / sub (net)</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Upfront commission (15%)</t>
         </is>
       </c>
       <c r="B13" s="9">
-        <f>((Assumptions!$B$5*0/100)+(Assumptions!$B$6*(1-0/100)))*12*(1-Assumptions!$B$9/100)</f>
+        <f>B7*Assumptions!$B$10/100</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>((Assumptions!$B$5*10/100)+(Assumptions!$B$6*(1-10/100)))*12*(1-Assumptions!$B$9/100)</f>
+        <f>C7*Assumptions!$B$10/100</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>((Assumptions!$B$5*20/100)+(Assumptions!$B$6*(1-20/100)))*12*(1-Assumptions!$B$9/100)</f>
+        <f>D7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="E13" s="9">
+        <f>E7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="F13" s="9">
+        <f>F7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="G13" s="9">
+        <f>G7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="H13" s="9">
+        <f>H7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="I13" s="9">
+        <f>I7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="J13" s="9">
+        <f>J7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="K13" s="9">
+        <f>K7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="L13" s="9">
+        <f>L7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="M13" s="9">
+        <f>M7*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="N13" s="9">
+        <f>SUM(B13:M13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Prepaid annual revenue (net)</t>
-        </is>
-      </c>
-      <c r="B14" s="9">
-        <f>Assumptions!$B$15*((Assumptions!$B$5*0/100)+(Assumptions!$B$6*(1-0/100)))*12*(1-Assumptions!$B$9/100)</f>
-        <v/>
-      </c>
-      <c r="C14" s="9">
-        <f>Assumptions!$B$15*((Assumptions!$B$5*10/100)+(Assumptions!$B$6*(1-10/100)))*12*(1-Assumptions!$B$9/100)</f>
-        <v/>
-      </c>
-      <c r="D14" s="9">
-        <f>Assumptions!$B$15*((Assumptions!$B$5*20/100)+(Assumptions!$B$6*(1-20/100)))*12*(1-Assumptions!$B$9/100)</f>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Year-end MSA bonus</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="9">
+        <f>Assumptions!$B$17*Assumptions!$B$11/100*Assumptions!$B$12/100</f>
+        <v/>
+      </c>
+      <c r="N14" s="9">
+        <f>SUM(B14:M14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Upfront commission (15%)</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Fixed opex (mktg/legal/sw/founder)</t>
         </is>
       </c>
       <c r="B15" s="9">
-        <f>(Assumptions!$B$15*((Assumptions!$B$5*0/100)+(Assumptions!$B$6*(1-0/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$10/100</f>
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
         <v/>
       </c>
       <c r="C15" s="9">
-        <f>(Assumptions!$B$15*((Assumptions!$B$5*10/100)+(Assumptions!$B$6*(1-10/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$10/100</f>
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
         <v/>
       </c>
       <c r="D15" s="9">
-        <f>(Assumptions!$B$15*((Assumptions!$B$5*20/100)+(Assumptions!$B$6*(1-20/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$10/100</f>
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="E15" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="F15" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="G15" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="H15" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="I15" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="J15" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="K15" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="L15" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="M15" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="N15" s="9">
+        <f>SUM(B15:M15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Year-end MSA bonus</t>
-        </is>
-      </c>
-      <c r="B16" s="9">
-        <f>(Assumptions!$B$15*((Assumptions!$B$5*0/100)+(Assumptions!$B$6*(1-0/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$11/100*Assumptions!$B$12/100</f>
-        <v/>
-      </c>
-      <c r="C16" s="9">
-        <f>(Assumptions!$B$15*((Assumptions!$B$5*10/100)+(Assumptions!$B$6*(1-10/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$11/100*Assumptions!$B$12/100</f>
-        <v/>
-      </c>
-      <c r="D16" s="9">
-        <f>(Assumptions!$B$15*((Assumptions!$B$5*20/100)+(Assumptions!$B$6*(1-20/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$11/100*Assumptions!$B$12/100</f>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Total operating expenses</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>B13+B14+B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="15">
+        <f>C13+C14+C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="15">
+        <f>D13+D14+D15</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>E13+E14+E15</f>
+        <v/>
+      </c>
+      <c r="F16" s="15">
+        <f>F13+F14+F15</f>
+        <v/>
+      </c>
+      <c r="G16" s="15">
+        <f>G13+G14+G15</f>
+        <v/>
+      </c>
+      <c r="H16" s="15">
+        <f>H13+H14+H15</f>
+        <v/>
+      </c>
+      <c r="I16" s="15">
+        <f>I13+I14+I15</f>
+        <v/>
+      </c>
+      <c r="J16" s="15">
+        <f>J13+J14+J15</f>
+        <v/>
+      </c>
+      <c r="K16" s="15">
+        <f>K13+K14+K15</f>
+        <v/>
+      </c>
+      <c r="L16" s="15">
+        <f>L13+L14+L15</f>
+        <v/>
+      </c>
+      <c r="M16" s="15">
+        <f>M13+M14+M15</f>
+        <v/>
+      </c>
+      <c r="N16" s="15">
+        <f>SUM(B16:M16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Total salesperson comp</t>
-        </is>
-      </c>
-      <c r="B17" s="13">
-        <f>B15+B16</f>
-        <v/>
-      </c>
-      <c r="C17" s="13">
-        <f>C15+C16</f>
-        <v/>
-      </c>
-      <c r="D17" s="13">
-        <f>D15+D16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Note: upfront commission is front-loaded cash at signing; the year-end bonus rewards 12-mo MSA completion (retention). Confirm plan mechanics with counsel/CPA.</t>
-        </is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>B12-B16</f>
+        <v/>
+      </c>
+      <c r="C17" s="15">
+        <f>C12-C16</f>
+        <v/>
+      </c>
+      <c r="D17" s="15">
+        <f>D12-D16</f>
+        <v/>
+      </c>
+      <c r="E17" s="15">
+        <f>E12-E16</f>
+        <v/>
+      </c>
+      <c r="F17" s="15">
+        <f>F12-F16</f>
+        <v/>
+      </c>
+      <c r="G17" s="15">
+        <f>G12-G16</f>
+        <v/>
+      </c>
+      <c r="H17" s="15">
+        <f>H12-H16</f>
+        <v/>
+      </c>
+      <c r="I17" s="15">
+        <f>I12-I16</f>
+        <v/>
+      </c>
+      <c r="J17" s="15">
+        <f>J12-J16</f>
+        <v/>
+      </c>
+      <c r="K17" s="15">
+        <f>K12-K16</f>
+        <v/>
+      </c>
+      <c r="L17" s="15">
+        <f>L12-L16</f>
+        <v/>
+      </c>
+      <c r="M17" s="15">
+        <f>M12-M16</f>
+        <v/>
+      </c>
+      <c r="N17" s="16">
+        <f>SUM(B17:M17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>EBITDA margin</t>
+        </is>
+      </c>
+      <c r="B18" s="14">
+        <f>IF(B7=0,0,B17/B7)</f>
+        <v/>
+      </c>
+      <c r="C18" s="14">
+        <f>IF(C7=0,0,C17/C7)</f>
+        <v/>
+      </c>
+      <c r="D18" s="14">
+        <f>IF(D7=0,0,D17/D7)</f>
+        <v/>
+      </c>
+      <c r="E18" s="14">
+        <f>IF(E7=0,0,E17/E7)</f>
+        <v/>
+      </c>
+      <c r="F18" s="14">
+        <f>IF(F7=0,0,F17/F7)</f>
+        <v/>
+      </c>
+      <c r="G18" s="14">
+        <f>IF(G7=0,0,G17/G7)</f>
+        <v/>
+      </c>
+      <c r="H18" s="14">
+        <f>IF(H7=0,0,H17/H7)</f>
+        <v/>
+      </c>
+      <c r="I18" s="14">
+        <f>IF(I7=0,0,I17/I7)</f>
+        <v/>
+      </c>
+      <c r="J18" s="14">
+        <f>IF(J7=0,0,J17/J7)</f>
+        <v/>
+      </c>
+      <c r="K18" s="14">
+        <f>IF(K7=0,0,K17/K7)</f>
+        <v/>
+      </c>
+      <c r="L18" s="14">
+        <f>IF(L7=0,0,L17/L7)</f>
+        <v/>
+      </c>
+      <c r="M18" s="14">
+        <f>IF(M7=0,0,M17/M7)</f>
+        <v/>
+      </c>
+      <c r="N18" s="14">
+        <f>IF(N7=0,0,N17/N7)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
@@ -1573,6 +2245,857 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>JHI Research &amp; Analytics Firm, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Monthly breakdown — accrual basis (ASC 606)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>generated 2026-07-19  ·  JHI-SIG: 69M2705M</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Revenue recognized ratably as cohorts stack; commission amortized over 12 mo. Builds monthly; the balance is deferred revenue carried to Yr 2 (see note).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>$ per month</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 1</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 2</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 3</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 4</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 5</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 6</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 7</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 8</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 9</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 10</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 11</t>
+        </is>
+      </c>
+      <c r="M5" s="12" t="inlineStr">
+        <is>
+          <t>Mo 12</t>
+        </is>
+      </c>
+      <c r="N5" s="12" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Recognized revenue</t>
+        </is>
+      </c>
+      <c r="B6" s="15">
+        <f>1*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="C6" s="15">
+        <f>2*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="D6" s="15">
+        <f>3*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>4*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="F6" s="15">
+        <f>5*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="G6" s="15">
+        <f>6*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="H6" s="15">
+        <f>7*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="I6" s="15">
+        <f>8*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="J6" s="15">
+        <f>9*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="K6" s="15">
+        <f>10*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="L6" s="15">
+        <f>11*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="M6" s="15">
+        <f>12*Assumptions!$B$8*Assumptions!$B$16/12</f>
+        <v/>
+      </c>
+      <c r="N6" s="15">
+        <f>SUM(B6:M6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total COGS</t>
+        </is>
+      </c>
+      <c r="B7" s="9">
+        <f>B6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="C7" s="9">
+        <f>C6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="D7" s="9">
+        <f>D6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="E7" s="9">
+        <f>E6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="F7" s="9">
+        <f>F6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="G7" s="9">
+        <f>G6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="H7" s="9">
+        <f>H6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="I7" s="9">
+        <f>I6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="J7" s="9">
+        <f>J6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="K7" s="9">
+        <f>K6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="L7" s="9">
+        <f>L6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="M7" s="9">
+        <f>M6*(Assumptions!$B$20+Assumptions!$B$21)/100+Assumptions!$B$22/12</f>
+        <v/>
+      </c>
+      <c r="N7" s="9">
+        <f>SUM(B7:M7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Gross profit</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
+        <f>B6-B7</f>
+        <v/>
+      </c>
+      <c r="C8" s="15">
+        <f>C6-C7</f>
+        <v/>
+      </c>
+      <c r="D8" s="15">
+        <f>D6-D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="15">
+        <f>E6-E7</f>
+        <v/>
+      </c>
+      <c r="F8" s="15">
+        <f>F6-F7</f>
+        <v/>
+      </c>
+      <c r="G8" s="15">
+        <f>G6-G7</f>
+        <v/>
+      </c>
+      <c r="H8" s="15">
+        <f>H6-H7</f>
+        <v/>
+      </c>
+      <c r="I8" s="15">
+        <f>I6-I7</f>
+        <v/>
+      </c>
+      <c r="J8" s="15">
+        <f>J6-J7</f>
+        <v/>
+      </c>
+      <c r="K8" s="15">
+        <f>K6-K7</f>
+        <v/>
+      </c>
+      <c r="L8" s="15">
+        <f>L6-L7</f>
+        <v/>
+      </c>
+      <c r="M8" s="15">
+        <f>M6-M7</f>
+        <v/>
+      </c>
+      <c r="N8" s="15">
+        <f>SUM(B8:M8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Commission (amortized)</t>
+        </is>
+      </c>
+      <c r="B9" s="9">
+        <f>1*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="C9" s="9">
+        <f>2*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="D9" s="9">
+        <f>3*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="E9" s="9">
+        <f>4*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="F9" s="9">
+        <f>5*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="G9" s="9">
+        <f>6*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="H9" s="9">
+        <f>7*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="I9" s="9">
+        <f>8*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="J9" s="9">
+        <f>9*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="K9" s="9">
+        <f>10*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="L9" s="9">
+        <f>11*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="M9" s="9">
+        <f>12*(Assumptions!$B$8*Assumptions!$B$16*Assumptions!$B$10/100)/12</f>
+        <v/>
+      </c>
+      <c r="N9" s="9">
+        <f>SUM(B9:M9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Fixed opex</t>
+        </is>
+      </c>
+      <c r="B10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="C10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="D10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="E10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="F10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="G10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="H10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="I10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="J10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="K10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="L10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="M10" s="9">
+        <f>(Assumptions!$B$23+Assumptions!$B$24+Assumptions!$B$25+Assumptions!$B$26)/12</f>
+        <v/>
+      </c>
+      <c r="N10" s="9">
+        <f>SUM(B10:M10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Year-end MSA bonus</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="9">
+        <f>Assumptions!$B$8*Assumptions!$B$11/100*Assumptions!$B$16*Assumptions!$B$12/100</f>
+        <v/>
+      </c>
+      <c r="N11" s="9">
+        <f>SUM(B11:M11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B12" s="15">
+        <f>B8-B9-B10-B11</f>
+        <v/>
+      </c>
+      <c r="C12" s="15">
+        <f>C8-C9-C10-C11</f>
+        <v/>
+      </c>
+      <c r="D12" s="15">
+        <f>D8-D9-D10-D11</f>
+        <v/>
+      </c>
+      <c r="E12" s="15">
+        <f>E8-E9-E10-E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="15">
+        <f>F8-F9-F10-F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="15">
+        <f>G8-G9-G10-G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="15">
+        <f>H8-H9-H10-H11</f>
+        <v/>
+      </c>
+      <c r="I12" s="15">
+        <f>I8-I9-I10-I11</f>
+        <v/>
+      </c>
+      <c r="J12" s="15">
+        <f>J8-J9-J10-J11</f>
+        <v/>
+      </c>
+      <c r="K12" s="15">
+        <f>K8-K9-K10-K11</f>
+        <v/>
+      </c>
+      <c r="L12" s="15">
+        <f>L8-L9-L10-L11</f>
+        <v/>
+      </c>
+      <c r="M12" s="15">
+        <f>M8-M9-M10-M11</f>
+        <v/>
+      </c>
+      <c r="N12" s="15">
+        <f>SUM(B12:M12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>EBITDA margin</t>
+        </is>
+      </c>
+      <c r="B13" s="14">
+        <f>IF(B6=0,0,B12/B6)</f>
+        <v/>
+      </c>
+      <c r="C13" s="14">
+        <f>IF(C6=0,0,C12/C6)</f>
+        <v/>
+      </c>
+      <c r="D13" s="14">
+        <f>IF(D6=0,0,D12/D6)</f>
+        <v/>
+      </c>
+      <c r="E13" s="14">
+        <f>IF(E6=0,0,E12/E6)</f>
+        <v/>
+      </c>
+      <c r="F13" s="14">
+        <f>IF(F6=0,0,F12/F6)</f>
+        <v/>
+      </c>
+      <c r="G13" s="14">
+        <f>IF(G6=0,0,G12/G6)</f>
+        <v/>
+      </c>
+      <c r="H13" s="14">
+        <f>IF(H6=0,0,H12/H6)</f>
+        <v/>
+      </c>
+      <c r="I13" s="14">
+        <f>IF(I6=0,0,I12/I6)</f>
+        <v/>
+      </c>
+      <c r="J13" s="14">
+        <f>IF(J6=0,0,J12/J6)</f>
+        <v/>
+      </c>
+      <c r="K13" s="14">
+        <f>IF(K6=0,0,K12/K6)</f>
+        <v/>
+      </c>
+      <c r="L13" s="14">
+        <f>IF(L6=0,0,L12/L6)</f>
+        <v/>
+      </c>
+      <c r="M13" s="14">
+        <f>IF(M6=0,0,M12/M6)</f>
+        <v/>
+      </c>
+      <c r="N13" s="14">
+        <f>IF(N6=0,0,N12/N6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Deferred to Yr 2 (booked − recognized):</t>
+        </is>
+      </c>
+      <c r="N15" s="9">
+        <f>Assumptions!$B$17-N6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Note: booked cash = full annual up front (see Bookings tab); accrual recognizes ratably, so Yr-1 EBITDA is lower but Yr 2 opens with revenue in hand.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;8© JHI Research &amp;&amp; Analytics Firm, Inc.  ·  JHI-SIG: 69M2705M&amp;C&amp;8Confidential — not for redistribution&amp;R&amp;8Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>JHI Research &amp; Analytics Firm, Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Salesperson total compensation &amp; mix sensitivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>generated 2026-07-19  ·  JHI-SIG: 69M2705M</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Upfront commission (15%)</t>
+        </is>
+      </c>
+      <c r="B5" s="15">
+        <f>'Upfront Commission (15%)'!$D$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Year-end MSA-completion bonus</t>
+        </is>
+      </c>
+      <c r="B6" s="15">
+        <f>'Year-End MSA Bonus'!$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Total salesperson compensation</t>
+        </is>
+      </c>
+      <c r="B7" s="13">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Total comp as % of revenue</t>
+        </is>
+      </c>
+      <c r="B8" s="14">
+        <f>IF(Assumptions!$B$17=0,0,B7/Assumptions!$B$17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Sensitivity — by Tier-1 mix (1,200 subs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>0% T1</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>10% T1</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>20% T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Avg full-paid price / sub (net)</t>
+        </is>
+      </c>
+      <c r="B13" s="9">
+        <f>((Assumptions!$B$5*0/100)+(Assumptions!$B$6*(1-0/100)))*12*(1-Assumptions!$B$9/100)</f>
+        <v/>
+      </c>
+      <c r="C13" s="9">
+        <f>((Assumptions!$B$5*10/100)+(Assumptions!$B$6*(1-10/100)))*12*(1-Assumptions!$B$9/100)</f>
+        <v/>
+      </c>
+      <c r="D13" s="9">
+        <f>((Assumptions!$B$5*20/100)+(Assumptions!$B$6*(1-20/100)))*12*(1-Assumptions!$B$9/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Prepaid annual revenue (net)</t>
+        </is>
+      </c>
+      <c r="B14" s="9">
+        <f>Assumptions!$B$15*((Assumptions!$B$5*0/100)+(Assumptions!$B$6*(1-0/100)))*12*(1-Assumptions!$B$9/100)</f>
+        <v/>
+      </c>
+      <c r="C14" s="9">
+        <f>Assumptions!$B$15*((Assumptions!$B$5*10/100)+(Assumptions!$B$6*(1-10/100)))*12*(1-Assumptions!$B$9/100)</f>
+        <v/>
+      </c>
+      <c r="D14" s="9">
+        <f>Assumptions!$B$15*((Assumptions!$B$5*20/100)+(Assumptions!$B$6*(1-20/100)))*12*(1-Assumptions!$B$9/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Upfront commission (15%)</t>
+        </is>
+      </c>
+      <c r="B15" s="9">
+        <f>(Assumptions!$B$15*((Assumptions!$B$5*0/100)+(Assumptions!$B$6*(1-0/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="C15" s="9">
+        <f>(Assumptions!$B$15*((Assumptions!$B$5*10/100)+(Assumptions!$B$6*(1-10/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+      <c r="D15" s="9">
+        <f>(Assumptions!$B$15*((Assumptions!$B$5*20/100)+(Assumptions!$B$6*(1-20/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$10/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Year-end MSA bonus</t>
+        </is>
+      </c>
+      <c r="B16" s="9">
+        <f>(Assumptions!$B$15*((Assumptions!$B$5*0/100)+(Assumptions!$B$6*(1-0/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$11/100*Assumptions!$B$12/100</f>
+        <v/>
+      </c>
+      <c r="C16" s="9">
+        <f>(Assumptions!$B$15*((Assumptions!$B$5*10/100)+(Assumptions!$B$6*(1-10/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$11/100*Assumptions!$B$12/100</f>
+        <v/>
+      </c>
+      <c r="D16" s="9">
+        <f>(Assumptions!$B$15*((Assumptions!$B$5*20/100)+(Assumptions!$B$6*(1-20/100)))*12*(1-Assumptions!$B$9/100))*Assumptions!$B$11/100*Assumptions!$B$12/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Total salesperson comp</t>
+        </is>
+      </c>
+      <c r="B17" s="13">
+        <f>B15+B16</f>
+        <v/>
+      </c>
+      <c r="C17" s="13">
+        <f>C15+C16</f>
+        <v/>
+      </c>
+      <c r="D17" s="13">
+        <f>D15+D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Note: upfront commission is front-loaded cash at signing; the year-end bonus rewards 12-mo MSA completion (retention). Confirm plan mechanics with counsel/CPA.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;8© JHI Research &amp;&amp; Analytics Firm, Inc.  ·  JHI-SIG: 69M2705M&amp;C&amp;8Confidential — not for redistribution&amp;R&amp;8Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>